<commit_message>
add department_id to User
</commit_message>
<xml_diff>
--- a/xlsx/Аббревиатуры подразделений.xlsx
+++ b/xlsx/Аббревиатуры подразделений.xlsx
@@ -914,18 +914,21 @@
       <color rgb="FF4D4D4D"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF4D4D4D"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF333333"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1202,7 +1205,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C141"/>
   <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="11.45" customHeight="true" zeroHeight="false" outlineLevelRow="3" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="85.94"/>
@@ -1241,7 +1244,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="4" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -1252,7 +1255,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="5" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -1263,7 +1266,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="6" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -1274,7 +1277,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="7" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>16</v>
       </c>
@@ -1285,7 +1288,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="8" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A8" s="4" t="s">
         <v>18</v>
       </c>
@@ -1296,7 +1299,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="9" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A9" s="4" t="s">
         <v>20</v>
       </c>
@@ -1307,7 +1310,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="10" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>22</v>
       </c>
@@ -1318,7 +1321,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="11" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A11" s="4" t="s">
         <v>24</v>
       </c>
@@ -1329,7 +1332,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="12" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A12" s="4" t="s">
         <v>26</v>
       </c>
@@ -1340,7 +1343,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="13" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A13" s="4" t="s">
         <v>28</v>
       </c>
@@ -1351,7 +1354,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="14" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A14" s="4" t="s">
         <v>30</v>
       </c>
@@ -1362,7 +1365,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="15" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A15" s="4" t="s">
         <v>32</v>
       </c>
@@ -1373,7 +1376,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="16" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A16" s="4" t="s">
         <v>34</v>
       </c>
@@ -1384,7 +1387,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="17" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A17" s="4" t="s">
         <v>36</v>
       </c>
@@ -1395,7 +1398,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="11" hidden="false" customHeight="true" outlineLevel="1" collapsed="false">
+    <row r="18" customFormat="false" ht="11" hidden="false" customHeight="true" outlineLevel="1" collapsed="true">
       <c r="A18" s="4" t="s">
         <v>38</v>
       </c>
@@ -2627,7 +2630,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="130" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="130" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A130" s="4" t="s">
         <v>261</v>
       </c>
@@ -2638,7 +2641,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="131" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="131" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A131" s="4" t="s">
         <v>263</v>
       </c>
@@ -2649,7 +2652,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="132" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="132" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A132" s="4" t="s">
         <v>265</v>
       </c>
@@ -2660,7 +2663,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="133" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="133" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A133" s="4" t="s">
         <v>267</v>
       </c>
@@ -2704,7 +2707,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="137" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="true">
+    <row r="137" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="true">
       <c r="A137" s="4" t="s">
         <v>275</v>
       </c>
@@ -2748,7 +2751,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="141" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="true">
+    <row r="141" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="true">
       <c r="A141" s="4" t="s">
         <v>283</v>
       </c>
@@ -2759,7 +2762,6 @@
         <v>284</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="11.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="true"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.39375" right="0.39375" top="0.39375" bottom="0.39375" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
add GDD for employee_schemas.py
</commit_message>
<xml_diff>
--- a/xlsx/Аббревиатуры подразделений.xlsx
+++ b/xlsx/Аббревиатуры подразделений.xlsx
@@ -1409,7 +1409,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="19" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>40</v>
       </c>
@@ -1420,7 +1420,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="20" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>42</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="21" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A21" s="4" t="s">
         <v>44</v>
       </c>
@@ -1442,7 +1442,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="11" hidden="false" customHeight="true" outlineLevel="1" collapsed="true">
+    <row r="22" customFormat="false" ht="11" hidden="false" customHeight="true" outlineLevel="1" collapsed="false">
       <c r="A22" s="4" t="s">
         <v>5</v>
       </c>
@@ -1453,7 +1453,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="23" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A23" s="4" t="s">
         <v>47</v>
       </c>
@@ -1464,7 +1464,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="24" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A24" s="4" t="s">
         <v>49</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="25" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A25" s="4" t="s">
         <v>51</v>
       </c>
@@ -1486,7 +1486,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="26" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A26" s="4" t="s">
         <v>53</v>
       </c>
@@ -1497,7 +1497,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="27" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="27" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>55</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="28" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A28" s="4" t="s">
         <v>57</v>
       </c>
@@ -1519,7 +1519,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="29" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A29" s="4" t="s">
         <v>59</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="2" collapsed="false">
+    <row r="30" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="2" collapsed="false">
       <c r="A30" s="4" t="s">
         <v>61</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="31" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A31" s="4" t="s">
         <v>63</v>
       </c>
@@ -1552,7 +1552,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="32" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A32" s="4" t="s">
         <v>65</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="33" s="1" customFormat="true" ht="11" hidden="true" customHeight="true" outlineLevel="3" collapsed="false">
+    <row r="33" s="1" customFormat="true" ht="11" hidden="false" customHeight="true" outlineLevel="3" collapsed="false">
       <c r="A33" s="4" t="s">
         <v>67</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="11" hidden="false" customHeight="true" outlineLevel="1" collapsed="true">
+    <row r="34" customFormat="false" ht="11" hidden="false" customHeight="true" outlineLevel="1" collapsed="false">
       <c r="A34" s="4" t="s">
         <v>69</v>
       </c>

</xml_diff>